<commit_message>
update DataGrouping6 notebook  & all excel DataGrouping6
</commit_message>
<xml_diff>
--- a/DataGrouping/ResultGrouping/hasil_klasifikasi_model6_Ryan.xlsx
+++ b/DataGrouping/ResultGrouping/hasil_klasifikasi_model6_Ryan.xlsx
@@ -19,17 +19,23 @@
     <sheet name="10_Balance_Terburuk" sheetId="10" r:id="rId10"/>
     <sheet name="10_PCA_Terbaik" sheetId="11" r:id="rId11"/>
     <sheet name="10_PCA_Terburuk" sheetId="12" r:id="rId12"/>
-    <sheet name="10_Normalisasi_Terbaik" sheetId="13" r:id="rId13"/>
-    <sheet name="10_Normalisasi_Terburuk" sheetId="14" r:id="rId14"/>
-    <sheet name="20_Terbaik_No_KFold" sheetId="15" r:id="rId15"/>
-    <sheet name="20_Terburuk_No_KFold" sheetId="16" r:id="rId16"/>
+    <sheet name="10_Norm_Terbaik" sheetId="13" r:id="rId13"/>
+    <sheet name="10_Norm_Terburuk" sheetId="14" r:id="rId14"/>
+    <sheet name="20_Terbaik_NoKFold" sheetId="15" r:id="rId15"/>
+    <sheet name="20_Terburuk_NoKFold" sheetId="16" r:id="rId16"/>
+    <sheet name="PCA_Terbaik_NoKFold" sheetId="17" r:id="rId17"/>
+    <sheet name="PCA_Terburuk_NoKFold" sheetId="18" r:id="rId18"/>
+    <sheet name="Balance_Terbaik_NoKFold" sheetId="19" r:id="rId19"/>
+    <sheet name="Balance_Terburuk_NoKFold" sheetId="20" r:id="rId20"/>
+    <sheet name="Norm_Terbaik_NoKFold" sheetId="21" r:id="rId21"/>
+    <sheet name="Norm_Terburuk_NoKFold" sheetId="22" r:id="rId22"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1144" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1498" uniqueCount="93">
   <si>
     <t>Percobaan</t>
   </si>
@@ -4193,6 +4199,1002 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="8" width="25.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.9675892206846322</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.9634421403428558</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.9613892681602998</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.962402075638082</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.9671036659383344</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.9632126948307868</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.9605940737206964</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.9618787376505152</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.9658897790725904</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.964261188894286</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.95737448690409</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.9607401367467509</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.9662539451323136</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.9643792699425422</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.9571815951079448</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.9606516401647508</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.9654042243262928</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.9626137601462964</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.9579824252609984</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.9602428237640768</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.9646758922068464</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.9606146032132152</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.958393399428522</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.9594955628425594</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.9645545035202721</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.960732950613806</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.957241864295684</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.9589558124143648</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.9632192279679532</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.961701828585692</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.9528697898333094</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0.957138887244768</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0.9627336732216556</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.960752247588196</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.9527165159373964</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0.9566132530275588</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.9620053411022093</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.95684665411928</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.9562871796534992</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0.9565652350558542</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="8" width="25.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.4547220199077446</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.419656611190381</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.2932406685641245</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.2701529030289784</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.4529011896091284</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.4136833697184386</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.3022389341437025</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.2749476148304676</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.4598203447438698</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.4499907211361029</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.3174447907921602</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.3034315851224228</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.4462248118475358</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.4598964289080941</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.3356765946275917</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.3161787696524699</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.4764505948045642</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.488325169173134</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.3262074108587348</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.3180408769870665</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.4697742170429716</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.4422739983739808</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.3660511021270397</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.3519026267549193</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.3869871327992231</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.3942720036822356</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.4212530967982199</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.3768243250940855</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.3882010196649672</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.3942358211841553</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.4227881731324888</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0.3779159658167711</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0.3908715707696042</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.3966917191931103</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.425322921691181</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0.3807191240539586</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.4792425345957756</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.4610120795607957</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.3860739690635166</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0.384313534972699</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="8" width="25.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.9861616897305172</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.9845296343674846</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.9836373717312272</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.9840748678948046</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.986404467103666</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.9844652037752226</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.9834278612770287</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.9839332854274758</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.9855547462976452</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.9839874511474987</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.9824300090310594</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.983196982747076</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.9853119689244962</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.9835859810899836</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.9825379553313358</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.9830525196960226</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.9851905802379218</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.9834530108886071</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.9824515745763416</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.9829430044491336</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.9854333576110706</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.9835728519203361</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.9819065131439551</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.9827258629347552</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.9851905802379218</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.9831676048150954</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.9822155348478891</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.9826863103185678</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.9853119689244962</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.9834002513905789</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.9818512100909536</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0.9826146115523664</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0.9848264141781986</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.9823478532750218</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.981749500045032</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0.9820388983088444</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.9845836368050498</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.9821429703423692</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.9817080570779332</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0.981922415653196</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I21"/>
@@ -4807,6 +5809,1002 @@
         <v>32</v>
       </c>
       <c r="I21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="8" width="25.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.3811604758436513</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.3914663150798229</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.4057841995367606</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.356951878548609</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.3811604758436513</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.3914663150798229</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.4057841995367606</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.356951878548609</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.3826171400825443</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.3927649012520344</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.4079233383404833</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.3591569896557414</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.3826171400825443</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.3927649012520344</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.4079233383404833</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.3591569896557414</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.3829813061422675</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.3945267522203496</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.4099137059552561</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.3604749977809582</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.3829813061422675</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.3945267522203496</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.4099137059552561</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.3604749977809582</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.3869871327992231</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.3942720036822356</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.4212530967982199</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.3768243250940855</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.3882010196649672</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.3942358211841553</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.4227881731324888</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0.3779159658167711</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0.3908715707696042</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.3966917191931103</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.425322921691181</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0.3807191240539586</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.3911143481427531</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.4162853968359508</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.4234606237110177</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0.3916114388990751</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="8" width="25.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.9855547462976452</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.9839874511474987</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.9824300090310594</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.983196982747076</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.9854333576110706</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.9844531313909756</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.9816334684432558</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.9830172074562959</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.9851905802379218</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.9834530108886071</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.9824515745763416</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.9829430044491336</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.9854333576110706</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.9835728519203361</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.9819065131439551</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.9827258629347552</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.9848264141781986</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.9840673506017972</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.9810756883297278</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.9825492540761086</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.9848264141781986</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.9823478532750218</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.981749500045032</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.9820388983088444</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.9845836368050498</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.9821429703423692</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.9817080570779332</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.981922415653196</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.984340859431901</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.9818254852241796</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.9813261680175128</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0.9815732294590352</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0.9840980820587522</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.9822550637355441</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.9808295153977412</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0.9815266563409</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.98349113862588</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.981787620530327</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.9800295612291507</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0.9808766411120254</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="8" width="25.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.4547220199077446</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.419656611190381</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.2932406685641245</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.2701529030289784</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.4529011896091284</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.4136833697184386</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.3022389341437025</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.2749476148304676</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.4598203447438698</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.4499907211361029</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.3174447907921602</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.3034315851224228</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.4462248118475358</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.4598964289080941</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.3356765946275917</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.3161787696524699</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.4764505948045642</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.488325169173134</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.3262074108587348</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.3180408769870665</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.4832483612527312</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.3783586099967141</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.3619857088142662</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.3373978529553924</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.4204904102937606</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.3573830887835812</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.3809224038259824</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.3448603757234413</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.4697742170429716</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.4422739983739808</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.3660511021270397</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0.3519026267549193</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0.3811604758436513</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.3914663150798229</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.4057841995367606</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0.356951878548609</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.3826171400825443</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.3927649012520344</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.4079233383404833</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0.3591569896557414</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>